<commit_message>
sel: halve side margins in PDF path (0.3 → 0.15)
Top/bottom/header/footer kept as is; only L/R cut to give fit-to-page
more printable width to work against. The padding columns A/U inside
print_area already keep column T on a single page, so wide side
margins are wasted ink.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/sel.xlsx
+++ b/template/sel.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\go\srmt-prime\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC6F78A-781D-4E2E-98AF-C78B04521D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9BBBABC-EF33-42BE-BC2E-7D413B000545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="252" yWindow="348" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Сухроб планшетга" sheetId="1" r:id="rId1"/>
+    <sheet name="list" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Сухроб планшетга'!$B$1:$U$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">list!$A$1:$U$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,10 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
-    <t>Ўзбекгидроэнерго АЖ бошқарувидаги сув омборларнинг хар соатлик амалда ишлаши тўғрисида тезкор
-Маълумот</t>
-  </si>
-  <si>
     <t>Т/р</t>
   </si>
   <si>
@@ -94,6 +90,9 @@
   </si>
   <si>
     <t>Вазиятлар маркази тезкор навбатчиси</t>
+  </si>
+  <si>
+    <t>Ўзбекгидроэнерго АЖ бошқарувидаги сув омборларнинг хар соатлик амалда ишлаши тўғрисида тезкор маълумот</t>
   </si>
 </sst>
 </file>
@@ -104,7 +103,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="[$-10819]hh:mm;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,35 +144,6 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
       <i/>
       <sz val="12"/>
       <name val="Times New Roman"/>
@@ -192,6 +162,64 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="16"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -436,7 +464,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -446,122 +474,128 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -880,274 +914,274 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:U11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="2.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="5.44140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.33203125" style="1" customWidth="1"/>
     <col min="4" max="5" width="10.109375" style="1" customWidth="1"/>
     <col min="6" max="17" width="8.5546875" style="1" customWidth="1"/>
     <col min="18" max="19" width="8.109375" style="1" customWidth="1"/>
     <col min="20" max="20" width="28.77734375" style="1" customWidth="1"/>
-    <col min="21" max="21" width="8.6640625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="2.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="22" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:21" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
-      <c r="S1" s="28"/>
-      <c r="T1" s="28"/>
+    <row r="1" spans="2:21" ht="53.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B1" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19"/>
+      <c r="T1" s="19"/>
     </row>
-    <row r="2" spans="2:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="16"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
-      <c r="T2" s="14">
+    <row r="2" spans="2:21" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="7"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="T2" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:21" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="T3" s="12">
+    <row r="3" spans="2:21" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="T3" s="9">
         <v>46140</v>
       </c>
-      <c r="U3" s="12"/>
+      <c r="U3" s="4"/>
     </row>
-    <row r="4" spans="2:21" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="37" t="s">
+    <row r="4" spans="2:21" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="31" t="s">
+      <c r="D4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="E4" s="23"/>
+      <c r="F4" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="23" t="s">
+      <c r="G4" s="23"/>
+      <c r="H4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="24"/>
-      <c r="H4" s="23" t="s">
+      <c r="I4" s="23"/>
+      <c r="J4" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="24"/>
-      <c r="J4" s="23" t="s">
+      <c r="K4" s="23"/>
+      <c r="L4" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="24"/>
-      <c r="L4" s="23" t="s">
+      <c r="M4" s="23"/>
+      <c r="N4" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="24"/>
-      <c r="N4" s="23" t="s">
+      <c r="O4" s="23"/>
+      <c r="P4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="O4" s="24"/>
-      <c r="P4" s="23" t="s">
+      <c r="Q4" s="23"/>
+      <c r="R4" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="24"/>
-      <c r="R4" s="23" t="s">
+      <c r="S4" s="23"/>
+      <c r="T4" s="20" t="s">
         <v>10</v>
-      </c>
-      <c r="S4" s="24"/>
-      <c r="T4" s="29" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="2:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="38"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="11">
+      <c r="B5" s="33"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="M5" s="11">
+      <c r="M5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="N5" s="11">
+      <c r="N5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="O5" s="11">
+      <c r="O5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="P5" s="11">
+      <c r="P5" s="10">
         <f>MOD($T$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="Q5" s="11">
+      <c r="Q5" s="10">
         <f>$T$2</f>
         <v>0</v>
       </c>
-      <c r="R5" s="10" t="s">
+      <c r="R5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="S5" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="T5" s="21"/>
+    </row>
+    <row r="6" spans="2:21" ht="49.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="38">
+        <v>1</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="30"/>
+      <c r="D6" s="12">
+        <v>0</v>
+      </c>
+      <c r="E6" s="13">
+        <v>0</v>
+      </c>
+      <c r="F6" s="14">
+        <v>0</v>
+      </c>
+      <c r="G6" s="15">
+        <v>0</v>
+      </c>
+      <c r="H6" s="14">
+        <v>0</v>
+      </c>
+      <c r="I6" s="16">
+        <v>0</v>
+      </c>
+      <c r="J6" s="14">
+        <v>0</v>
+      </c>
+      <c r="K6" s="15">
+        <v>0</v>
+      </c>
+      <c r="L6" s="17">
+        <v>0</v>
+      </c>
+      <c r="M6" s="16">
+        <v>0</v>
+      </c>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="17">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="15">
+        <v>0</v>
+      </c>
+      <c r="R6" s="36"/>
+      <c r="S6" s="36"/>
+      <c r="T6" s="28"/>
     </row>
-    <row r="6" spans="2:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="21">
-        <v>1</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="9">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7">
-        <v>0</v>
-      </c>
-      <c r="I6" s="6">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7">
-        <v>0</v>
-      </c>
-      <c r="K6" s="4">
-        <v>0</v>
-      </c>
-      <c r="L6" s="5">
-        <v>0</v>
-      </c>
-      <c r="M6" s="6">
-        <v>0</v>
-      </c>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4">
-        <v>0</v>
-      </c>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="33"/>
-    </row>
-    <row r="7" spans="2:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="22"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="25">
+    <row r="7" spans="2:21" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="39"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="24">
         <f>IFERROR(E6-D6, "-")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="26"/>
-      <c r="F7" s="25">
+      <c r="E7" s="25"/>
+      <c r="F7" s="24">
         <f>IFERROR(G6-F6, "-")</f>
         <v>0</v>
       </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="25">
+      <c r="G7" s="25"/>
+      <c r="H7" s="24">
         <f>IFERROR(I6-H6, "-")</f>
         <v>0</v>
       </c>
-      <c r="I7" s="26"/>
-      <c r="J7" s="25">
+      <c r="I7" s="25"/>
+      <c r="J7" s="24">
         <f>IFERROR(K6-J6, "-")</f>
         <v>0</v>
       </c>
-      <c r="K7" s="26"/>
-      <c r="L7" s="25">
+      <c r="K7" s="25"/>
+      <c r="L7" s="24">
         <f>IFERROR(M6-L6, "-")</f>
         <v>0</v>
       </c>
-      <c r="M7" s="26"/>
-      <c r="N7" s="25">
+      <c r="M7" s="25"/>
+      <c r="N7" s="24">
         <f>IFERROR(O6-N6, "-")</f>
         <v>0</v>
       </c>
-      <c r="O7" s="26"/>
-      <c r="P7" s="25">
+      <c r="O7" s="25"/>
+      <c r="P7" s="24">
         <f>IFERROR(Q6-P6, "-")</f>
         <v>0</v>
       </c>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
-      <c r="T7" s="34"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="37"/>
+      <c r="S7" s="37"/>
+      <c r="T7" s="29"/>
     </row>
     <row r="8" spans="2:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="2:21" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1155,21 +1189,21 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
+      <c r="F9" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="35"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="18"/>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
     </row>
@@ -1179,6 +1213,16 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="F9:K9"/>
+    <mergeCell ref="S6:S7"/>
+    <mergeCell ref="N9:R9"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="R6:R7"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="P7:Q7"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="T4:T5"/>
     <mergeCell ref="H4:I4"/>
@@ -1195,19 +1239,9 @@
     <mergeCell ref="N7:O7"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F9:K9"/>
-    <mergeCell ref="S6:S7"/>
-    <mergeCell ref="N9:R9"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="R6:R7"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="P7:Q7"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0" bottom="0" header="0.11811023622047249" footer="0.11811023622047249"/>
-  <pageSetup paperSize="9" scale="71" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="74" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sel/generator: rely on template style for row-5 prev (no SetCellStyle)
The previous version applied NewStyle({NumFmt: 49}) + SetCellStyle to the
row-5 prev cells to force text format. That wiped every other style
attribute carried by the template (alignment, wrap-text, borders, font),
which broke the visual layout: cells lost centering and the multi-line
hh:mm subheader rendered without wrap.

Fix: trust the template. The .xlsx now carries text format + wrap-text on
C5/E5/G5/I5/K5/M5/O5 directly, so SetCellValue with a string preserves
both style and content. The NumFmt:49-driven dance was needed only when
the template still claimed [$-10819]hh:mm;@ for those cells.

Template (template/sel.xlsx) updated to ship the correct cell style.
</commit_message>
<xml_diff>
--- a/template/sel.xlsx
+++ b/template/sel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\go\srmt-prime\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A7ED40-D602-48B9-9885-06DA82F2BE01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235F45CB-AC62-4C7D-9803-2C58D43BAF2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="252" yWindow="348" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="list" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Т/р</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>Ўзбекгидроэнерго АЖ бошқарувидаги сув омборларнинг хар соатлик амалда ишлаши тўғрисида тезкор маълумот</t>
+  </si>
+  <si>
+    <t>12:00 - 14:00</t>
   </si>
 </sst>
 </file>
@@ -488,7 +491,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -549,61 +552,6 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="167" fontId="9" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -619,12 +567,70 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -957,27 +963,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="53.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
     </row>
     <row r="2" spans="1:19" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6"/>
@@ -1010,103 +1016,102 @@
       </c>
     </row>
     <row r="4" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="26" t="s">
+      <c r="A4" s="40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="22" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="23"/>
-      <c r="G4" s="22" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="23"/>
-      <c r="I4" s="22" t="s">
+      <c r="H4" s="25"/>
+      <c r="I4" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="23"/>
-      <c r="K4" s="22" t="s">
+      <c r="J4" s="25"/>
+      <c r="K4" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="23"/>
-      <c r="M4" s="22" t="s">
+      <c r="L4" s="25"/>
+      <c r="M4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="N4" s="23"/>
-      <c r="O4" s="22" t="s">
+      <c r="N4" s="25"/>
+      <c r="O4" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="22" t="s">
+      <c r="P4" s="25"/>
+      <c r="Q4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="R4" s="23"/>
-      <c r="S4" s="20" t="s">
+      <c r="R4" s="25"/>
+      <c r="S4" s="32" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="9">
+    <row r="5" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="41"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="9">
+        <f>$S$2</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="42">
         <f>MOD($S$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="D5" s="9">
+      <c r="F5" s="9">
         <f>$S$2</f>
         <v>0</v>
       </c>
-      <c r="E5" s="9">
+      <c r="G5" s="42">
         <f>MOD($S$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="F5" s="9">
+      <c r="H5" s="9">
         <f>$S$2</f>
         <v>0</v>
       </c>
-      <c r="G5" s="9">
+      <c r="I5" s="42">
         <f>MOD($S$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="H5" s="9">
+      <c r="J5" s="9">
         <f>$S$2</f>
         <v>0</v>
       </c>
-      <c r="I5" s="9">
+      <c r="K5" s="42">
         <f>MOD($S$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="J5" s="9">
+      <c r="L5" s="9">
         <f>$S$2</f>
         <v>0</v>
       </c>
-      <c r="K5" s="9">
+      <c r="M5" s="42">
         <f>MOD($S$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="L5" s="9">
+      <c r="N5" s="9">
         <f>$S$2</f>
         <v>0</v>
       </c>
-      <c r="M5" s="9">
+      <c r="O5" s="42">
         <f>MOD($S$2-TIME(1,0,0),1)</f>
         <v>0.95833333333333337</v>
       </c>
-      <c r="N5" s="9">
-        <f>$S$2</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="9">
-        <f>MOD($S$2-TIME(1,0,0),1)</f>
-        <v>0.95833333333333337</v>
-      </c>
       <c r="P5" s="9">
         <f>$S$2</f>
         <v>0</v>
@@ -1117,13 +1122,13 @@
       <c r="R5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="S5" s="21"/>
+      <c r="S5" s="33"/>
     </row>
     <row r="6" spans="1:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="38">
+      <c r="A6" s="22">
         <v>1</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="38" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="11">
@@ -1164,73 +1169,73 @@
       <c r="P6" s="14">
         <v>0</v>
       </c>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="34"/>
-      <c r="S6" s="28"/>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="36"/>
     </row>
     <row r="7" spans="1:19" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="39"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="24">
+      <c r="A7" s="23"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="26">
         <f>IFERROR(D6-C6, "-")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="24">
+      <c r="D7" s="27"/>
+      <c r="E7" s="26">
         <f>IFERROR(F6-E6, "-")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="25"/>
-      <c r="G7" s="24">
+      <c r="F7" s="27"/>
+      <c r="G7" s="26">
         <f>IFERROR(H6-G6, "-")</f>
         <v>0</v>
       </c>
-      <c r="H7" s="25"/>
-      <c r="I7" s="24">
+      <c r="H7" s="27"/>
+      <c r="I7" s="26">
         <f>IFERROR(J6-I6, "-")</f>
         <v>0</v>
       </c>
-      <c r="J7" s="25"/>
-      <c r="K7" s="24">
+      <c r="J7" s="27"/>
+      <c r="K7" s="26">
         <f>IFERROR(L6-K6, "-")</f>
         <v>0</v>
       </c>
-      <c r="L7" s="25"/>
-      <c r="M7" s="24">
+      <c r="L7" s="27"/>
+      <c r="M7" s="26">
         <f>IFERROR(N6-M6, "-")</f>
         <v>0</v>
       </c>
-      <c r="N7" s="25"/>
-      <c r="O7" s="24">
+      <c r="N7" s="27"/>
+      <c r="O7" s="26">
         <f>IFERROR(P6-O6, "-")</f>
         <v>0</v>
       </c>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="35"/>
-      <c r="S7" s="29"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="29"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="37"/>
     </row>
     <row r="8" spans="1:19" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
       <c r="L9" s="17"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
+      <c r="M9" s="20"/>
+      <c r="N9" s="21"/>
+      <c r="O9" s="21"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
     </row>
@@ -1240,16 +1245,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="R6:R7"/>
-    <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="Q6:Q7"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="C9:K9"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="S4:S5"/>
     <mergeCell ref="G4:H4"/>
@@ -1266,6 +1261,16 @@
     <mergeCell ref="M7:N7"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="R6:R7"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="Q6:Q7"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="C9:K9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0" bottom="0" header="0.11811023622047249" footer="0.11811023622047249"/>

</xml_diff>